<commit_message>
global wave add feb26
</commit_message>
<xml_diff>
--- a/global_wave.xlsx
+++ b/global_wave.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\factor_system\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\factor-platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F176F033-89B0-41DB-9DEF-A8B61F19B919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D0442D-0B19-497C-8565-B55642B1281B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4302" yWindow="3696" windowWidth="17280" windowHeight="9984" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -82,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,6 +101,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -370,8 +382,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15.3" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="9.234375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
@@ -483,6 +498,11 @@
       </c>
       <c r="B14" s="2">
         <v>45757</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="3">
+        <v>46069</v>
       </c>
     </row>
   </sheetData>

</xml_diff>